<commit_message>
Strip HTML from RSS excerpts (found in a live end-to-end run)
Ran a real research job end-to-end ('what people on Discord/Kick/Twitch are
saying about the new Spider-Man movie'). The engine planned the job, reported
Twitch/Kick/Discord as unconfigured with working fallbacks, collected 8 real
articles via RSS, built the dossier, and exported all five files.

The live run exposed a data-quality bug unit tests missed: feeds that put HTML
in their summary field (Google News search feeds return <a> tags) were stored
as raw markup, so evidence excerpts were unreadable. Added _plain_text() to
reduce feed HTML to readable text and applied it to the RSS title, excerpt, and
author. Excerpts are now clean headlines.

Logged as F4 in docs/FEATURE_STATUS.xlsx. 99 Python + 16 extension tests pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FiGhdqEHy4JuVT6JWdeY4F
</commit_message>
<xml_diff>
--- a/docs/FEATURE_STATUS.xlsx
+++ b/docs/FEATURE_STATUS.xlsx
@@ -45,7 +45,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +97,11 @@
         <fgColor rgb="00F8D7DA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCEFC7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,6 +167,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -783,11 +791,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
+      <c r="K4" s="15" t="inlineStr">
+        <is>
+          <t>F4 (data quality, found in live Spider-Man run): feed summaries with HTML (e.g. Google News) were stored as raw &lt;a&gt; markup instead of readable text.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Added _plain_text() to strip tags + unescape entities; applied to RSS title/excerpt/author.</t>
+        </is>
+      </c>
       <c r="M4" s="13" t="inlineStr">
         <is>
-          <t>PASS (re-verified green)</t>
+          <t>PASS (live re-run shows clean headlines; test_feed_html_is_reduced_to_readable_text)</t>
         </is>
       </c>
     </row>
@@ -6210,7 +6226,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
@@ -6311,8 +6326,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>

</xml_diff>